<commit_message>
feat(dashboard): group all 19 system functions into operational flow tabs and verify button execution
</commit_message>
<xml_diff>
--- a/IPO-applied.xlsx
+++ b/IPO-applied.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.44140625" customWidth="1" min="1" max="1"/>
@@ -486,6 +486,22 @@
       </c>
       <c r="D3" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Moneyview  Pric</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5632</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-77.90384956167323</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-438754.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): update operational applied records, user log tracks, and master sync
</commit_message>
<xml_diff>
--- a/IPO-applied.xlsx
+++ b/IPO-applied.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.44140625" customWidth="1" min="1" max="1"/>
@@ -495,14 +495,20 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5632</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>-77.90384956167323</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>-438754.48</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -515,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.44140625" customWidth="1" min="1" max="1"/>
@@ -562,6 +568,22 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Moneyview  Pric</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5632</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-77.90384956167323</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-438754.48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: record latest live application audit trail
</commit_message>
<xml_diff>
--- a/IPO-applied.xlsx
+++ b/IPO-applied.xlsx
@@ -508,7 +508,6 @@
           <t>APPLIED</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -521,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.44140625" customWidth="1" min="1" max="1"/>
@@ -575,13 +574,23 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5632</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>-77.90384956167323</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>-438754.48</v>
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>OTP not received</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: remove test/fake IPO records; keep only real Excel-matched IPOs
- IPO-applied.xlsx: removed 'Beta Mainboard IPO' (test record)
- capitalfund.db ipo_applied table: deleted ids 1,2,3
  (Test Automation IPO, Alpha SME IPO, Beta Mainboard IPO) via
  scratch/cleanup_test_ipos.py fuzzy-matched against General.xlsx
- Remaining records: Moneyview (APPLIED uci=1, FAILED uci=2)
  which are real IPOs present in General.xlsx IPOMB
</commit_message>
<xml_diff>
--- a/IPO-applied.xlsx
+++ b/IPO-applied.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.44140625" customWidth="1" min="1" max="1"/>
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.44140625" customWidth="1" min="1" max="1"/>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Beta Mainboard IPO</t>
+          <t>Moneyview  Pric</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -566,28 +566,12 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Moneyview  Pric</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>FAILED</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>OTP not received</t>
         </is>

</xml_diff>